<commit_message>
chore: cleanup procedural artifacts and update operational files
- Removed obsolete procedural level files (procedural_d_slot2.json, progression_ dir, slot2_4.json)
- Updated memoria.md with 2026-04-13 migration summary
- Updated package.json dependencies
- Updated spreadsheet sync and Google Sheets reconnect scripts
- Refreshed level report generation script
</commit_message>
<xml_diff>
--- a/minigame_locally/minigames/Levels_feed_the_bear_after_feedback_sync.xlsx
+++ b/minigame_locally/minigames/Levels_feed_the_bear_after_feedback_sync.xlsx
@@ -5035,6 +5035,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
@@ -5278,7 +5279,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>02 · progresion1 level2</t>
+          <t>02 · progression1 level2</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -5293,7 +5294,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>progresion1_level2.json</t>
+          <t>progression1_level2.json</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -5446,7 +5447,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>06 · progresion1 level6</t>
+          <t>06 · progression1 level6</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -5461,7 +5462,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>progresion1_level6.json</t>
+          <t>progression1_level6.json</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -5703,7 +5704,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>01 · progresion2 level1</t>
+          <t>01 · progression2 level1</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -5718,7 +5719,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>progresion2_level1.json</t>
+          <t>progression2_level1.json</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -5745,7 +5746,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>02 · progresion2 level2</t>
+          <t>02 · progression2 level2</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -5760,7 +5761,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>progresion2_level2.json</t>
+          <t>progression2_level2.json</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -5787,7 +5788,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>03 · progresion2 level3</t>
+          <t>03 · progression2 level3</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -5802,7 +5803,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>progresion2_level3.json</t>
+          <t>progression2_level3.json</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -5829,7 +5830,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>04 · progresion2 level4</t>
+          <t>04 · progression2 level4</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -5844,7 +5845,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>progresion2_level4.json</t>
+          <t>progression2_level4.json</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -5871,7 +5872,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>05 · progresion2 level5</t>
+          <t>05 · progression2 level5</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -5886,7 +5887,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>progresion2_level5.json</t>
+          <t>progression2_level5.json</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -5913,7 +5914,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>06 · progresion2 level6</t>
+          <t>06 · progression2 level6</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -5928,7 +5929,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>progresion2_level6.json</t>
+          <t>progression2_level6.json</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -5955,7 +5956,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>07 · progresion2 level7</t>
+          <t>07 · progression2 level7</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -5970,7 +5971,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>progresion2_level7.json</t>
+          <t>progression2_level7.json</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -5997,7 +5998,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>08 · progresion2 level8</t>
+          <t>08 · progression2 level8</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -6012,7 +6013,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>progresion2_level8.json</t>
+          <t>progression2_level8.json</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -6039,7 +6040,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>09 · progresion2 level9</t>
+          <t>09 · progression2 level9</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -6054,7 +6055,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>progresion2_level9.json</t>
+          <t>progression2_level9.json</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -6081,7 +6082,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>10 · progresion2 level10</t>
+          <t>10 · progression2 level10</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -6096,7 +6097,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>progresion2_level10.json</t>
+          <t>progression2_level10.json</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -11430,7 +11431,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>progresion1_level2.json</t>
+          <t>progression1_level2.json</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -11450,7 +11451,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>progresion1_level6.json</t>
+          <t>progression1_level6.json</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -11496,7 +11497,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>progresion1_level2.png</t>
+          <t>progression1_level2.png</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -11516,7 +11517,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>progresion1_level6.png</t>
+          <t>progression1_level6.png</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -11640,7 +11641,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>progresion1_level2.json</t>
+          <t>progression1_level2.json</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -11660,7 +11661,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>progresion1_level6.json</t>
+          <t>progression1_level6.json</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -11706,7 +11707,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>progresion1_level2.png</t>
+          <t>progression1_level2.png</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -11726,7 +11727,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>progresion1_level6.png</t>
+          <t>progression1_level6.png</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -11855,52 +11856,52 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>progresion2_level1.json</t>
+          <t>progression2_level1.json</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>progresion2_level2.json</t>
+          <t>progression2_level2.json</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>progresion2_level3.json</t>
+          <t>progression2_level3.json</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>progresion2_level4.json</t>
+          <t>progression2_level4.json</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>progresion2_level5.json</t>
+          <t>progression2_level5.json</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>progresion2_level6.json</t>
+          <t>progression2_level6.json</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>progresion2_level7.json</t>
+          <t>progression2_level7.json</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>progresion2_level8.json</t>
+          <t>progression2_level8.json</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>progresion2_level9.json</t>
+          <t>progression2_level9.json</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>progresion2_level10.json</t>
+          <t>progression2_level10.json</t>
         </is>
       </c>
       <c r="R8">
@@ -11921,52 +11922,52 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>progresion2_level1.png</t>
+          <t>progression2_level1.png</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>progresion2_level2.png</t>
+          <t>progression2_level2.png</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>progresion2_level3.png</t>
+          <t>progression2_level3.png</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>progresion2_level4.png</t>
+          <t>progression2_level4.png</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>progresion2_level5.png</t>
+          <t>progression2_level5.png</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>progresion2_level6.png</t>
+          <t>progression2_level6.png</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>progresion2_level7.png</t>
+          <t>progression2_level7.png</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>progresion2_level8.png</t>
+          <t>progression2_level8.png</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>progresion2_level9.png</t>
+          <t>progression2_level9.png</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>progresion2_level10.png</t>
+          <t>progression2_level10.png</t>
         </is>
       </c>
     </row>
@@ -12070,52 +12071,52 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>progresion2_level2.json</t>
+          <t>progression2_level2.json</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>progresion2_level3.json</t>
+          <t>progression2_level3.json</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>progresion2_level4.json</t>
+          <t>progression2_level4.json</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>progresion2_level5.json</t>
+          <t>progression2_level5.json</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>progresion2_level6.json</t>
+          <t>progression2_level6.json</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>progresion2_level7.json</t>
+          <t>progression2_level7.json</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>progresion2_level8.json</t>
+          <t>progression2_level8.json</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>progresion2_level9.json</t>
+          <t>progression2_level9.json</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>progresion2_level10.json</t>
+          <t>progression2_level10.json</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>progresion2_level1.json</t>
+          <t>progression2_level1.json</t>
         </is>
       </c>
       <c r="R11">
@@ -12136,52 +12137,52 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>progresion2_level2.png</t>
+          <t>progression2_level2.png</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>progresion2_level3.png</t>
+          <t>progression2_level3.png</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>progresion2_level4.png</t>
+          <t>progression2_level4.png</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>progresion2_level5.png</t>
+          <t>progression2_level5.png</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>progresion2_level6.png</t>
+          <t>progression2_level6.png</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>progresion2_level7.png</t>
+          <t>progression2_level7.png</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>progresion2_level8.png</t>
+          <t>progression2_level8.png</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>progresion2_level9.png</t>
+          <t>progression2_level9.png</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>progresion2_level10.png</t>
+          <t>progression2_level10.png</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>progresion2_level1.png</t>
+          <t>progression2_level1.png</t>
         </is>
       </c>
     </row>
@@ -17020,7 +17021,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>progresion2_level2.json</t>
+          <t>progression2_level2.json</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -17086,7 +17087,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>progresion2_level2.png</t>
+          <t>progression2_level2.png</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -17230,7 +17231,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>progresion2_level1.json</t>
+          <t>progression2_level1.json</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -17296,7 +17297,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>progresion2_level1.png</t>
+          <t>progression2_level1.png</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -17822,37 +17823,37 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>progresion1 level2</t>
+          <t>progression1 level2</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>02 · progresion1 level2</t>
+          <t>02 · progression1 level2</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>progresion1_level2.json</t>
+          <t>progression1_level2.json</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion1_level2.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression1_level2.json</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>progresion1_level2.png</t>
+          <t>progression1_level2.png</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progresion1_level2.png</t>
+          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progression1_level2.png</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>progresion1_level2.json</t>
+          <t>progression1_level2.json</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -18070,37 +18071,37 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>progresion1 level6</t>
+          <t>progression1 level6</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>06 · progresion1 level6</t>
+          <t>06 · progression1 level6</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>progresion1_level6.json</t>
+          <t>progression1_level6.json</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion1_level6.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression1_level6.json</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>progresion1_level6.png</t>
+          <t>progression1_level6.png</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progresion1_level6.png</t>
+          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progression1_level6.png</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>progresion1_level6.json</t>
+          <t>progression1_level6.json</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -18380,37 +18381,37 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>progresion2 level1</t>
+          <t>progression2 level1</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>01 · progresion2 level1</t>
+          <t>01 · progression2 level1</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>progresion2_level1.json</t>
+          <t>progression2_level1.json</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level1.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level1.json</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>progresion2_level1.png</t>
+          <t>progression2_level1.png</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progresion2_level1.png</t>
+          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progression2_level1.png</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>progresion2_level1.json</t>
+          <t>progression2_level1.json</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -18442,37 +18443,37 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>progresion2 level2</t>
+          <t>progression2 level2</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>02 · progresion2 level2</t>
+          <t>02 · progression2 level2</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>progresion2_level2.json</t>
+          <t>progression2_level2.json</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level2.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level2.json</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>progresion2_level2.png</t>
+          <t>progression2_level2.png</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progresion2_level2.png</t>
+          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progression2_level2.png</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>progresion2_level2.json</t>
+          <t>progression2_level2.json</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -18504,37 +18505,37 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>progresion2 level3</t>
+          <t>progression2 level3</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>03 · progresion2 level3</t>
+          <t>03 · progression2 level3</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>progresion2_level3.json</t>
+          <t>progression2_level3.json</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level3.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level3.json</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>progresion2_level3.png</t>
+          <t>progression2_level3.png</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progresion2_level3.png</t>
+          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progression2_level3.png</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>progresion2_level3.json</t>
+          <t>progression2_level3.json</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -18566,37 +18567,37 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>progresion2 level4</t>
+          <t>progression2 level4</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>04 · progresion2 level4</t>
+          <t>04 · progression2 level4</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>progresion2_level4.json</t>
+          <t>progression2_level4.json</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level4.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level4.json</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>progresion2_level4.png</t>
+          <t>progression2_level4.png</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progresion2_level4.png</t>
+          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progression2_level4.png</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>progresion2_level4.json</t>
+          <t>progression2_level4.json</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -18628,37 +18629,37 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>progresion2 level5</t>
+          <t>progression2 level5</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>05 · progresion2 level5</t>
+          <t>05 · progression2 level5</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>progresion2_level5.json</t>
+          <t>progression2_level5.json</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level5.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level5.json</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>progresion2_level5.png</t>
+          <t>progression2_level5.png</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progresion2_level5.png</t>
+          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progression2_level5.png</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>progresion2_level5.json</t>
+          <t>progression2_level5.json</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -18690,37 +18691,37 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>progresion2 level6</t>
+          <t>progression2 level6</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>06 · progresion2 level6</t>
+          <t>06 · progression2 level6</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>progresion2_level6.json</t>
+          <t>progression2_level6.json</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level6.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level6.json</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>progresion2_level6.png</t>
+          <t>progression2_level6.png</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progresion2_level6.png</t>
+          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progression2_level6.png</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>progresion2_level6.json</t>
+          <t>progression2_level6.json</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -18752,37 +18753,37 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>progresion2 level7</t>
+          <t>progression2 level7</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>07 · progresion2 level7</t>
+          <t>07 · progression2 level7</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>progresion2_level7.json</t>
+          <t>progression2_level7.json</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level7.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level7.json</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>progresion2_level7.png</t>
+          <t>progression2_level7.png</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progresion2_level7.png</t>
+          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progression2_level7.png</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>progresion2_level7.json</t>
+          <t>progression2_level7.json</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -18814,37 +18815,37 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>progresion2 level8</t>
+          <t>progression2 level8</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>08 · progresion2 level8</t>
+          <t>08 · progression2 level8</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>progresion2_level8.json</t>
+          <t>progression2_level8.json</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level8.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level8.json</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>progresion2_level8.png</t>
+          <t>progression2_level8.png</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progresion2_level8.png</t>
+          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progression2_level8.png</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>progresion2_level8.json</t>
+          <t>progression2_level8.json</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -18876,37 +18877,37 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>progresion2 level9</t>
+          <t>progression2 level9</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>09 · progresion2 level9</t>
+          <t>09 · progression2 level9</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>progresion2_level9.json</t>
+          <t>progression2_level9.json</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level9.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level9.json</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>progresion2_level9.png</t>
+          <t>progression2_level9.png</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progresion2_level9.png</t>
+          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progression2_level9.png</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>progresion2_level9.json</t>
+          <t>progression2_level9.json</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -18938,37 +18939,37 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>progresion2 level10</t>
+          <t>progression2 level10</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>10 · progresion2 level10</t>
+          <t>10 · progression2 level10</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>progresion2_level10.json</t>
+          <t>progression2_level10.json</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level10.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level10.json</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>progresion2_level10.png</t>
+          <t>progression2_level10.png</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progresion2_level10.png</t>
+          <t>/sessions/bold-affectionate-fermi/mnt/minigame_locally/levels/screenshots/progression2_level10.png</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>progresion2_level10.json</t>
+          <t>progression2_level10.json</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -26027,12 +26028,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>progresion1_level2.json</t>
+          <t>progression1_level2.json</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>progresion1 level2</t>
+          <t>progression1 level2</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -26075,12 +26076,12 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>progresion1_level2.png</t>
+          <t>progression1_level2.png</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion1_level2.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression1_level2.json</t>
         </is>
       </c>
       <c r="M4" s="10" t="inlineStr">
@@ -26287,12 +26288,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>progresion1_level6.json</t>
+          <t>progression1_level6.json</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>progresion1 level6</t>
+          <t>progression1 level6</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -26335,12 +26336,12 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>progresion1_level6.png</t>
+          <t>progression1_level6.png</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion1_level6.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression1_level6.json</t>
         </is>
       </c>
       <c r="M8" s="10" t="inlineStr">
@@ -26612,12 +26613,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>progresion2_level1.json</t>
+          <t>progression2_level1.json</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>progresion2 level1</t>
+          <t>progression2 level1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -26660,12 +26661,12 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>progresion2_level1.png</t>
+          <t>progression2_level1.png</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level1.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level1.json</t>
         </is>
       </c>
       <c r="M13" s="10" t="inlineStr">
@@ -26677,12 +26678,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>progresion2_level2.json</t>
+          <t>progression2_level2.json</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>progresion2 level2</t>
+          <t>progression2 level2</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -26725,12 +26726,12 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>progresion2_level2.png</t>
+          <t>progression2_level2.png</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level2.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level2.json</t>
         </is>
       </c>
       <c r="M14" s="10" t="inlineStr">
@@ -26742,12 +26743,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>progresion2_level3.json</t>
+          <t>progression2_level3.json</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>progresion2 level3</t>
+          <t>progression2 level3</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -26790,12 +26791,12 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>progresion2_level3.png</t>
+          <t>progression2_level3.png</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level3.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level3.json</t>
         </is>
       </c>
       <c r="M15" s="10" t="inlineStr">
@@ -26807,12 +26808,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>progresion2_level4.json</t>
+          <t>progression2_level4.json</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>progresion2 level4</t>
+          <t>progression2 level4</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -26855,12 +26856,12 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>progresion2_level4.png</t>
+          <t>progression2_level4.png</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level4.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level4.json</t>
         </is>
       </c>
       <c r="M16" s="10" t="inlineStr">
@@ -26872,12 +26873,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>progresion2_level5.json</t>
+          <t>progression2_level5.json</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>progresion2 level5</t>
+          <t>progression2 level5</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -26920,12 +26921,12 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>progresion2_level5.png</t>
+          <t>progression2_level5.png</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level5.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level5.json</t>
         </is>
       </c>
       <c r="M17" s="10" t="inlineStr">
@@ -26937,12 +26938,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>progresion2_level6.json</t>
+          <t>progression2_level6.json</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>progresion2 level6</t>
+          <t>progression2 level6</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -26985,12 +26986,12 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>progresion2_level6.png</t>
+          <t>progression2_level6.png</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level6.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level6.json</t>
         </is>
       </c>
       <c r="M18" s="10" t="inlineStr">
@@ -27002,12 +27003,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>progresion2_level7.json</t>
+          <t>progression2_level7.json</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>progresion2 level7</t>
+          <t>progression2 level7</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -27050,12 +27051,12 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>progresion2_level7.png</t>
+          <t>progression2_level7.png</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level7.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level7.json</t>
         </is>
       </c>
       <c r="M19" s="11" t="inlineStr">
@@ -27067,12 +27068,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>progresion2_level8.json</t>
+          <t>progression2_level8.json</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>progresion2 level8</t>
+          <t>progression2 level8</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -27115,12 +27116,12 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>progresion2_level8.png</t>
+          <t>progression2_level8.png</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level8.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level8.json</t>
         </is>
       </c>
       <c r="M20" s="11" t="inlineStr">
@@ -27132,12 +27133,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>progresion2_level9.json</t>
+          <t>progression2_level9.json</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>progresion2 level9</t>
+          <t>progression2 level9</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -27180,12 +27181,12 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>progresion2_level9.png</t>
+          <t>progression2_level9.png</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level9.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level9.json</t>
         </is>
       </c>
       <c r="M21" s="11" t="inlineStr">
@@ -27197,12 +27198,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>progresion2_level10.json</t>
+          <t>progression2_level10.json</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>progresion2 level10</t>
+          <t>progression2 level10</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -27245,12 +27246,12 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>progresion2_level10.png</t>
+          <t>progression2_level10.png</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level10.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level10.json</t>
         </is>
       </c>
       <c r="M22" s="11" t="inlineStr">
@@ -34734,12 +34735,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>progresion1_level2.json</t>
+          <t>progression1_level2.json</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>progresion1 level2</t>
+          <t>progression1 level2</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -34779,12 +34780,12 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>minigame_locally/levels/progresion1_level2.json</t>
+          <t>minigame_locally/levels/progression1_level2.json</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion1_level2.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression1_level2.json</t>
         </is>
       </c>
       <c r="S4" s="10" t="inlineStr">
@@ -35062,12 +35063,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>progresion1_level6.json</t>
+          <t>progression1_level6.json</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>progresion1 level6</t>
+          <t>progression1 level6</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -35107,12 +35108,12 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>minigame_locally/levels/progresion1_level6.json</t>
+          <t>minigame_locally/levels/progression1_level6.json</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion1_level6.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression1_level6.json</t>
         </is>
       </c>
       <c r="S8" s="10" t="inlineStr">
@@ -35559,12 +35560,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>progresion2_level1.json</t>
+          <t>progression2_level1.json</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>progresion2 level1</t>
+          <t>progression2 level1</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -35604,12 +35605,12 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>minigame_locally/levels/progresion2_level1.json</t>
+          <t>minigame_locally/levels/progression2_level1.json</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level1.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level1.json</t>
         </is>
       </c>
       <c r="S14" s="10" t="inlineStr">
@@ -35641,12 +35642,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>progresion2_level2.json</t>
+          <t>progression2_level2.json</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>progresion2 level2</t>
+          <t>progression2 level2</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -35686,12 +35687,12 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>minigame_locally/levels/progresion2_level2.json</t>
+          <t>minigame_locally/levels/progression2_level2.json</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level2.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level2.json</t>
         </is>
       </c>
       <c r="S15" s="10" t="inlineStr">
@@ -35723,12 +35724,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>progresion2_level3.json</t>
+          <t>progression2_level3.json</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>progresion2 level3</t>
+          <t>progression2 level3</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -35768,12 +35769,12 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>minigame_locally/levels/progresion2_level3.json</t>
+          <t>minigame_locally/levels/progression2_level3.json</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level3.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level3.json</t>
         </is>
       </c>
       <c r="S16" s="10" t="inlineStr">
@@ -35805,12 +35806,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>progresion2_level4.json</t>
+          <t>progression2_level4.json</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>progresion2 level4</t>
+          <t>progression2 level4</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -35850,12 +35851,12 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>minigame_locally/levels/progresion2_level4.json</t>
+          <t>minigame_locally/levels/progression2_level4.json</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level4.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level4.json</t>
         </is>
       </c>
       <c r="S17" s="10" t="inlineStr">
@@ -35887,12 +35888,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>progresion2_level5.json</t>
+          <t>progression2_level5.json</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>progresion2 level5</t>
+          <t>progression2 level5</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -35932,12 +35933,12 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>minigame_locally/levels/progresion2_level5.json</t>
+          <t>minigame_locally/levels/progression2_level5.json</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level5.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level5.json</t>
         </is>
       </c>
       <c r="S18" s="10" t="inlineStr">
@@ -35969,12 +35970,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>progresion2_level6.json</t>
+          <t>progression2_level6.json</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>progresion2 level6</t>
+          <t>progression2 level6</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -36014,12 +36015,12 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>minigame_locally/levels/progresion2_level6.json</t>
+          <t>minigame_locally/levels/progression2_level6.json</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level6.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level6.json</t>
         </is>
       </c>
       <c r="S19" s="10" t="inlineStr">
@@ -36051,12 +36052,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>progresion2_level7.json</t>
+          <t>progression2_level7.json</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>progresion2 level7</t>
+          <t>progression2 level7</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -36096,12 +36097,12 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>minigame_locally/levels/progresion2_level7.json</t>
+          <t>minigame_locally/levels/progression2_level7.json</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level7.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level7.json</t>
         </is>
       </c>
       <c r="S20" s="11" t="inlineStr">
@@ -36133,12 +36134,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>progresion2_level8.json</t>
+          <t>progression2_level8.json</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>progresion2 level8</t>
+          <t>progression2 level8</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -36178,12 +36179,12 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>minigame_locally/levels/progresion2_level8.json</t>
+          <t>minigame_locally/levels/progression2_level8.json</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level8.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level8.json</t>
         </is>
       </c>
       <c r="S21" s="11" t="inlineStr">
@@ -36215,12 +36216,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>progresion2_level9.json</t>
+          <t>progression2_level9.json</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>progresion2 level9</t>
+          <t>progression2 level9</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -36260,12 +36261,12 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>minigame_locally/levels/progresion2_level9.json</t>
+          <t>minigame_locally/levels/progression2_level9.json</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level9.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level9.json</t>
         </is>
       </c>
       <c r="S22" s="11" t="inlineStr">
@@ -36297,12 +36298,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>progresion2_level10.json</t>
+          <t>progression2_level10.json</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>progresion2 level10</t>
+          <t>progression2 level10</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -36342,12 +36343,12 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>minigame_locally/levels/progresion2_level10.json</t>
+          <t>minigame_locally/levels/progression2_level10.json</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progresion2_level10.json</t>
+          <t>/Users/victoria.serrano/Library/CloudStorage/SynologyDrive-back1/misScripts/minigame_locally/levels/progression2_level10.json</t>
         </is>
       </c>
       <c r="S23" s="11" t="inlineStr">

</xml_diff>